<commit_message>
Marketing 23.09. 10:30: Fahrten im Kanalplan auf 0 EUR (Deutschlandticket), sieben erfundene Merkmal-Zeilen aus der Preiskarte entfernt
- gtm-kanalplan.xlsx: Kanal x Monat!D11 200 -> 120 EUR (2 Dessau-Fahrten
  entfallen, Deutschlandticket). Annahmen F2/F6/A13/A14 mit Begruendung,
  neuen Summen (1.350 EUR) und neuer Vorsteuer (181,62 EUR).
  Die 360 EUR fuer kalte Laeden ab Apr 27 bleiben bewusst stehen.
- PreiseSection: die sieben Haekchen-Zeilen standen nicht im freigegebenen
  Landingpage-Entwurf und widersprachen der Merkmals-Sektion darueber
  ("Export" statt "direkt", DATEV fehlte). Entfernt, Abstand ausgeglichen.
- Ergebnisse in der eigenen Datei, Zahlen an Finance, Fund an Engineering.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MFg2T2cAFiNYZJYBD1wJD6
</commit_message>
<xml_diff>
--- a/docs/gtm-kanalplan.xlsx
+++ b/docs/gtm-kanalplan.xlsx
@@ -737,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="30" min="1" max="1"/>
@@ -820,7 +820,7 @@
       </c>
       <c r="F2" s="36" t="inlineStr">
         <is>
-          <t>Okt: Druck Flyer+Aufsteller ~120 €, 2 Fahrten ~80 € · danach ~20 €/Monat. ALLE Betraege BRUTTO (Endpreis inkl. USt). Druck 19 %. Fahrten = Bahn Berlin&lt;&gt;Dessau, RE7 direkt, ~20 € je Richtung, 7 % (Personenbefoerderung Schienenbahn, § 12 Abs. 2 Nr. 10 UStG).</t>
+          <t>Okt: Druck Flyer+Aufsteller ~120 EUR, 2 Fahrten 0 EUR (Deutschlandticket) · danach ~20 EUR/Monat. ALLE Betraege BRUTTO (Endpreis inkl. USt). Druck 19 %. Fahrten Berlin&lt;&gt;Dessau: RE7 direkt, Nahverkehr - abgedeckt durch Sandys Deutschlandticket, das sie fuer ihren Angestelltenjob ohnehin haelt (Sandys Antwort, 23.09.2026). Keine zusaetzlichen Kosten, keine Vorsteuer. Als Tagesfahrten geplant, keine Uebernachtungszeile.</t>
         </is>
       </c>
       <c r="G2" s="36" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="F6" s="36" t="inlineStr">
         <is>
-          <t>Pro Laden ~60 € Druck + ~40 € Fahrt. BRUTTO. Druck 19 %, Fahrt = Bahn, 7 %.</t>
+          <t>Pro Laden ~60 EUR Druck + ~40 EUR Fahrt. BRUTTO. Druck 19 %, Fahrt = Bahn, 7 %. Fahrt hier bewusst NICHT auf 0 gesetzt, obwohl Sandy ein Deutschlandticket hat: dieser Kanal startet erst Apr 27, das Ticket haengt an ihrem Angestelltenjob, und welche Laeden es werden, steht nicht fest (ausserhalb des Nahverkehrs waere es ein eigener Fahrschein).</t>
         </is>
       </c>
       <c r="G6" s="36" t="inlineStr">
@@ -1086,7 +1086,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="15" customHeight="1" s="31">
       <c r="A10" s="37" t="inlineStr">
         <is>
@@ -1101,11 +1100,17 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="30" t="inlineStr">
         <is>
-          <t>Hinweis Marketing (23.09.2026): Alle Sachkosten-Groessenordnungen auf diesem Blatt sind BRUTTO gemeint, also der Betrag, der vom Konto geht. Nicht netto. Steuersaetze: Druck/Ausruestung/Kleinbedarf 19 %, Fahrten 7 % (Bahn). Vorsteuer ueber 24 Monate daraus: 186,85 €.</t>
+          <t>Hinweis Marketing (23.09.2026, 2. Fassung): Alle Sachkosten-Groessenordnungen auf diesem Blatt sind BRUTTO gemeint, also der Betrag, der vom Konto geht. Nicht netto. Steuersaetze: Druck/Ausruestung/Kleinbedarf 19 %, Fahrten 7 % (Bahn, § 12 Abs. 2 Nr. 10 UStG). Geaendert am 23.09.2026: die zwei Dessau-Fahrten im Okt 26 (80 EUR) stehen auf 0 EUR, weil Sandys Deutschlandticket sie abdeckt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Sachkosten 24 Monate: 1.350 EUR (vorher 1.430 EUR). Aufschluesselung: Druck 660 EUR · Fahrten 360 EUR (nur noch kalte Laeden ab Apr 27) · Ausruestung 60 EUR · Kleinbedarf 270 EUR. Vorsteuer daraus: 181,62 EUR (vorher 186,85 EUR). Mischsatz 0,1345323176. Die Zahl im Finanzplan (Plan-Kosten AL47/AM47) setzt Finance, nicht Marketing.</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1859,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="46" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="E11" s="46" t="n">
         <v>0</v>

</xml_diff>